<commit_message>
Add employee business tests, trim project_staffing to the spec
- pandera rejects an employee reporting to themselves
- dbt singular tests mirror the loader's row-level rules (status/termination,
  termination after hire, no self-reporting) as errors; inactive manager warns
- lead-rank uniqueness test guards the ranking window in int_project_leads
- project_staffing drops active_lead_count; multi-lead warning moves to intermediate
- README: duplicates policy, severity rule of thumb, test table
</commit_message>
<xml_diff>
--- a/data/hr_employees_export_invalid.xlsx
+++ b/data/hr_employees_export_invalid.xlsx
@@ -883,6 +883,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>EMP-1007</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">

</xml_diff>